<commit_message>
Update latest raw objectives
</commit_message>
<xml_diff>
--- a/latest_raw/futgg_raw_objectives_latest.xlsx
+++ b/latest_raw/futgg_raw_objectives_latest.xlsx
@@ -488,7 +488,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 03:55:04</t>
+          <t>2026-09-16 04:57:58</t>
         </is>
       </c>
     </row>
@@ -500,7 +500,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 02:00:00</t>
+          <t>2026-09-16 02:00:00</t>
         </is>
       </c>
     </row>

</xml_diff>